<commit_message>
Add measurement units to template headers + insect severity column
Client requested units shown on the deliverable and a dedicated insect
severity rating.

- Bake units into both template headers (the source of truth, so every
  export shows them): TDR °C / dS/m / %, tissue macros %, micros ppm.
- Add Insect_Damage_Severity (Low/Med/High) after Insect_Damage in both
  templates; generalize the classifier so any *_Severity is a severity field.
- Introduce a unit-stripped Field.key so classification, nutrient/severity
  pairing, the form's TDR lookups, and importer column matching stay
  unit-agnostic while names/DB columns/exports carry the unit text.

Verified end-to-end: classify, pairing, obs schema, lab-column auto-map
(N -> "N (%)"), save round-trip, and Excel + GPKG export for both crops.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Static Canola Template.xlsx
+++ b/Static Canola Template.xlsx
@@ -120,7 +120,7 @@
     <xf numFmtId="0" fontId="1" fillId="8" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="9" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="2"/>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="3"/>
@@ -135,6 +135,7 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="9">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -540,7 +541,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:CE10"/>
+  <dimension ref="A1:CF10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
     <col width="3.265625" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -572,7 +573,7 @@
     <col width="13" bestFit="1" customWidth="1" min="30" max="30"/>
     <col width="24.19921875" bestFit="1" customWidth="1" min="31" max="31"/>
     <col width="13.53125" bestFit="1" customWidth="1" min="32" max="32"/>
-    <col width="17.796875" bestFit="1" customWidth="1" min="33" max="33"/>
+    <col width="13.53125" bestFit="1" customWidth="1" min="33" max="33"/>
     <col width="8.59765625" bestFit="1" customWidth="1" min="34" max="34"/>
     <col width="2.19921875" bestFit="1" customWidth="1" min="35" max="35"/>
     <col width="6.19921875" bestFit="1" customWidth="1" min="36" max="36"/>
@@ -648,47 +649,47 @@
       </c>
       <c r="E1" s="2" t="inlineStr">
         <is>
-          <t>TDR_1_SOIL_TEMPERATURE</t>
+          <t>TDR_1_SOIL_TEMPERATURE (°C)</t>
         </is>
       </c>
       <c r="F1" s="2" t="inlineStr">
         <is>
-          <t>TDR_1_SOIL_EC</t>
+          <t>TDR_1_SOIL_EC (dS/m)</t>
         </is>
       </c>
       <c r="G1" s="2" t="inlineStr">
         <is>
-          <t>TDR_1_SOIL_MOISTURE</t>
+          <t>TDR_1_SOIL_MOISTURE (%)</t>
         </is>
       </c>
       <c r="H1" s="2" t="inlineStr">
         <is>
-          <t>TDR_2_SOIL_TEMPERATURE</t>
+          <t>TDR_2_SOIL_TEMPERATURE (°C)</t>
         </is>
       </c>
       <c r="I1" s="2" t="inlineStr">
         <is>
-          <t>TDR_2_SOIL_EC</t>
+          <t>TDR_2_SOIL_EC (dS/m)</t>
         </is>
       </c>
       <c r="J1" s="2" t="inlineStr">
         <is>
-          <t>TDR_2_SOIL_MOISTURE</t>
+          <t>TDR_2_SOIL_MOISTURE (%)</t>
         </is>
       </c>
       <c r="K1" s="2" t="inlineStr">
         <is>
-          <t>TDR_3_SOIL_TEMPERATURE</t>
+          <t>TDR_3_SOIL_TEMPERATURE (°C)</t>
         </is>
       </c>
       <c r="L1" s="2" t="inlineStr">
         <is>
-          <t>TDR_3_SOIL_EC</t>
+          <t>TDR_3_SOIL_EC (dS/m)</t>
         </is>
       </c>
       <c r="M1" s="2" t="inlineStr">
         <is>
-          <t>TDR_3_SOIL_MOISTURE</t>
+          <t>TDR_3_SOIL_MOISTURE (%)</t>
         </is>
       </c>
       <c r="N1" s="3" t="inlineStr">
@@ -786,257 +787,262 @@
           <t>Insect_Damage</t>
         </is>
       </c>
-      <c r="AG1" s="6" t="inlineStr">
+      <c r="AG1" s="10" t="inlineStr">
+        <is>
+          <t>Insect_Damage_Severity</t>
+        </is>
+      </c>
+      <c r="AH1" s="6" t="inlineStr">
         <is>
           <t>Insect_Identification</t>
         </is>
       </c>
-      <c r="AH1" s="7" t="inlineStr">
+      <c r="AI1" s="7" t="inlineStr">
         <is>
           <t>ReportNo</t>
         </is>
       </c>
-      <c r="AI1" s="8" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
       <c r="AJ1" s="8" t="inlineStr">
         <is>
+          <t>N (%)</t>
+        </is>
+      </c>
+      <c r="AK1" s="8" t="inlineStr">
+        <is>
           <t>N_rate</t>
         </is>
       </c>
-      <c r="AK1" s="8" t="inlineStr">
-        <is>
-          <t>NO3N</t>
-        </is>
-      </c>
       <c r="AL1" s="8" t="inlineStr">
         <is>
+          <t>NO3N (ppm)</t>
+        </is>
+      </c>
+      <c r="AM1" s="8" t="inlineStr">
+        <is>
           <t>NO3N_rate</t>
         </is>
       </c>
-      <c r="AM1" s="8" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
       <c r="AN1" s="8" t="inlineStr">
         <is>
+          <t>P (%)</t>
+        </is>
+      </c>
+      <c r="AO1" s="8" t="inlineStr">
+        <is>
           <t>P_rate</t>
         </is>
       </c>
-      <c r="AO1" s="8" t="inlineStr">
-        <is>
-          <t>K</t>
-        </is>
-      </c>
       <c r="AP1" s="8" t="inlineStr">
         <is>
+          <t>K (%)</t>
+        </is>
+      </c>
+      <c r="AQ1" s="8" t="inlineStr">
+        <is>
           <t>K_rate</t>
         </is>
       </c>
-      <c r="AQ1" s="8" t="inlineStr">
-        <is>
-          <t>Ca</t>
-        </is>
-      </c>
       <c r="AR1" s="8" t="inlineStr">
         <is>
+          <t>Ca (%)</t>
+        </is>
+      </c>
+      <c r="AS1" s="8" t="inlineStr">
+        <is>
           <t>Ca_rate</t>
         </is>
       </c>
-      <c r="AS1" s="8" t="inlineStr">
-        <is>
-          <t>Mg</t>
-        </is>
-      </c>
       <c r="AT1" s="8" t="inlineStr">
         <is>
+          <t>Mg (%)</t>
+        </is>
+      </c>
+      <c r="AU1" s="8" t="inlineStr">
+        <is>
           <t>Mg_rate</t>
         </is>
       </c>
-      <c r="AU1" s="8" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
-      </c>
       <c r="AV1" s="8" t="inlineStr">
         <is>
+          <t>S (%)</t>
+        </is>
+      </c>
+      <c r="AW1" s="8" t="inlineStr">
+        <is>
           <t>S_rate</t>
         </is>
       </c>
-      <c r="AW1" s="8" t="inlineStr">
-        <is>
-          <t>Zn</t>
-        </is>
-      </c>
       <c r="AX1" s="8" t="inlineStr">
         <is>
+          <t>Zn (ppm)</t>
+        </is>
+      </c>
+      <c r="AY1" s="8" t="inlineStr">
+        <is>
           <t>Zn_rate</t>
         </is>
       </c>
-      <c r="AY1" s="8" t="inlineStr">
-        <is>
-          <t>Mn</t>
-        </is>
-      </c>
       <c r="AZ1" s="8" t="inlineStr">
         <is>
+          <t>Mn (ppm)</t>
+        </is>
+      </c>
+      <c r="BA1" s="8" t="inlineStr">
+        <is>
           <t>Mn_rate</t>
         </is>
       </c>
-      <c r="BA1" s="8" t="inlineStr">
-        <is>
-          <t>Fe</t>
-        </is>
-      </c>
       <c r="BB1" s="8" t="inlineStr">
         <is>
+          <t>Fe (ppm)</t>
+        </is>
+      </c>
+      <c r="BC1" s="8" t="inlineStr">
+        <is>
           <t>Fe_rate</t>
         </is>
       </c>
-      <c r="BC1" s="8" t="inlineStr">
-        <is>
-          <t>Cu</t>
-        </is>
-      </c>
       <c r="BD1" s="8" t="inlineStr">
         <is>
+          <t>Cu (ppm)</t>
+        </is>
+      </c>
+      <c r="BE1" s="8" t="inlineStr">
+        <is>
           <t>Cu_rate</t>
         </is>
       </c>
-      <c r="BE1" s="8" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
       <c r="BF1" s="8" t="inlineStr">
         <is>
+          <t>B (ppm)</t>
+        </is>
+      </c>
+      <c r="BG1" s="8" t="inlineStr">
+        <is>
           <t>B_rate</t>
         </is>
       </c>
-      <c r="BG1" s="8" t="inlineStr">
-        <is>
-          <t>Mo</t>
-        </is>
-      </c>
       <c r="BH1" s="8" t="inlineStr">
         <is>
+          <t>Mo (ppm)</t>
+        </is>
+      </c>
+      <c r="BI1" s="8" t="inlineStr">
+        <is>
           <t>Mo_rate</t>
         </is>
       </c>
-      <c r="BI1" s="8" t="inlineStr">
-        <is>
-          <t>Al</t>
-        </is>
-      </c>
       <c r="BJ1" s="8" t="inlineStr">
         <is>
+          <t>Al (ppm)</t>
+        </is>
+      </c>
+      <c r="BK1" s="8" t="inlineStr">
+        <is>
           <t>Al_rate</t>
         </is>
       </c>
-      <c r="BK1" s="8" t="inlineStr">
-        <is>
-          <t>Na</t>
-        </is>
-      </c>
       <c r="BL1" s="8" t="inlineStr">
         <is>
+          <t>Na (%)</t>
+        </is>
+      </c>
+      <c r="BM1" s="8" t="inlineStr">
+        <is>
           <t>Na_rate</t>
         </is>
       </c>
-      <c r="BM1" s="8" t="inlineStr">
-        <is>
-          <t>Cl</t>
-        </is>
-      </c>
       <c r="BN1" s="8" t="inlineStr">
         <is>
+          <t>Cl (%)</t>
+        </is>
+      </c>
+      <c r="BO1" s="8" t="inlineStr">
+        <is>
           <t>Cl_rate</t>
         </is>
       </c>
-      <c r="BO1" s="8" t="inlineStr">
+      <c r="BP1" s="8" t="inlineStr">
         <is>
           <t>N/S_Actual</t>
         </is>
       </c>
-      <c r="BP1" s="8" t="inlineStr">
+      <c r="BQ1" s="8" t="inlineStr">
         <is>
           <t>N/S_Expected</t>
         </is>
       </c>
-      <c r="BQ1" s="8" t="inlineStr">
+      <c r="BR1" s="8" t="inlineStr">
         <is>
           <t>N/K_Actual</t>
         </is>
       </c>
-      <c r="BR1" s="8" t="inlineStr">
+      <c r="BS1" s="8" t="inlineStr">
         <is>
           <t>N/K_Expected</t>
         </is>
       </c>
-      <c r="BS1" s="8" t="inlineStr">
+      <c r="BT1" s="8" t="inlineStr">
         <is>
           <t>P/S_Actual</t>
         </is>
       </c>
-      <c r="BT1" s="8" t="inlineStr">
+      <c r="BU1" s="8" t="inlineStr">
         <is>
           <t>P/S_Expected</t>
         </is>
       </c>
-      <c r="BU1" s="8" t="inlineStr">
+      <c r="BV1" s="8" t="inlineStr">
         <is>
           <t>P/Zn_Actual</t>
         </is>
       </c>
-      <c r="BV1" s="8" t="inlineStr">
+      <c r="BW1" s="8" t="inlineStr">
         <is>
           <t>P/Zn_Expected</t>
         </is>
       </c>
-      <c r="BW1" s="8" t="inlineStr">
+      <c r="BX1" s="8" t="inlineStr">
         <is>
           <t>K/Mg_Actual</t>
         </is>
       </c>
-      <c r="BX1" s="8" t="inlineStr">
+      <c r="BY1" s="8" t="inlineStr">
         <is>
           <t>K/Mg_Expected</t>
         </is>
       </c>
-      <c r="BY1" s="8" t="inlineStr">
+      <c r="BZ1" s="8" t="inlineStr">
         <is>
           <t>K/Mn_Actual</t>
         </is>
       </c>
-      <c r="BZ1" s="8" t="inlineStr">
+      <c r="CA1" s="8" t="inlineStr">
         <is>
           <t>K/Mn_Expected</t>
         </is>
       </c>
-      <c r="CA1" s="8" t="inlineStr">
+      <c r="CB1" s="8" t="inlineStr">
         <is>
           <t>Ca/B_Actual</t>
         </is>
       </c>
-      <c r="CB1" s="8" t="inlineStr">
+      <c r="CC1" s="8" t="inlineStr">
         <is>
           <t>Ca/B_Expected</t>
         </is>
       </c>
-      <c r="CC1" s="8" t="inlineStr">
+      <c r="CD1" s="8" t="inlineStr">
         <is>
           <t>Fe/Mn_Actual</t>
         </is>
       </c>
-      <c r="CD1" s="8" t="inlineStr">
+      <c r="CE1" s="8" t="inlineStr">
         <is>
           <t>Fe/Mn_Expected</t>
         </is>
       </c>
-      <c r="CE1" s="9" t="inlineStr">
+      <c r="CF1" s="9" t="inlineStr">
         <is>
           <t>Images</t>
         </is>

</xml_diff>